<commit_message>
Add all Shirazi translations
</commit_message>
<xml_diff>
--- a/datasets/100_samples_shirazi.xlsx
+++ b/datasets/100_samples_shirazi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Personal Projects\SilkRoadNLP\Repositories\General\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E0B76B3-8331-4CD1-92EA-DC4509F07812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA537B3C-BD87-4126-A5F3-0A8D5D9C0D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="334">
   <si>
     <t>100_samples</t>
   </si>
@@ -1047,9 +1047,6 @@
     <t>ما عَم میویم.</t>
   </si>
   <si>
-    <t>دس بجنبون</t>
-  </si>
-  <si>
     <t>پس کجویی عزیزُم؟</t>
   </si>
   <si>
@@ -1071,9 +1068,6 @@
     <t>قدوی سرت. عیبی نداره.</t>
   </si>
   <si>
-    <t>آفتاب از کدوم سمت درومده؟ / امروز کُجُ دس و رومه شسّه بودم؟</t>
-  </si>
-  <si>
     <t>خانوم بچه‌ها چیطورن؟</t>
   </si>
   <si>
@@ -1108,6 +1102,129 @@
   </si>
   <si>
     <t>گربُو ره بُراق کِرده.</t>
+  </si>
+  <si>
+    <t>امروز کُجُ دس و رومه شسّه بودم؟</t>
+  </si>
+  <si>
+    <t>اَی امر حضرت حق نباشه، برگ از درخت نَمیوفته.</t>
+  </si>
+  <si>
+    <t>اَی نخوردیم نونِ گندم، ولی دیدیم دسِّ مردم.</t>
+  </si>
+  <si>
+    <t>جار</t>
+  </si>
+  <si>
+    <t>خسّه</t>
+  </si>
+  <si>
+    <t>بوگو چقدر حال می‌ده</t>
+  </si>
+  <si>
+    <t>لعنت به پدرت</t>
+  </si>
+  <si>
+    <t>هکروی ما از هکروی دیگه چیزی کم ندارن</t>
+  </si>
+  <si>
+    <t>خیلی جالب می‌شه</t>
+  </si>
+  <si>
+    <t>فقط وُیسو برِی یکی از بازیوی باحالت</t>
+  </si>
+  <si>
+    <t>ما برِی تازه‌ترین آتیش منتظر می‌مونیم</t>
+  </si>
+  <si>
+    <t>یعنی ساخته نمی‌شه</t>
+  </si>
+  <si>
+    <t>با ایکه ده تو کارگر داره،‌ پونزده سال طول می‌کشه</t>
+  </si>
+  <si>
+    <t>مِثکه کسوی دیگه‌ای هم با هواپیما به لوگر می‌رن</t>
+  </si>
+  <si>
+    <t>ساختن ای فرودگاهو هم عین رفتن به ماعه</t>
+  </si>
+  <si>
+    <t>درخت میوه کرم از خودشه</t>
+  </si>
+  <si>
+    <t>بیرون باغُ که دیدیم، انگو تا تَهِ باغُ دیدیم.</t>
+  </si>
+  <si>
+    <t>حرفه اَی داخل شیشه کنی به بیرون درز می‌کنه.</t>
+  </si>
+  <si>
+    <t>حرف تا وقتی تو دلته اختیارش دسِّته.</t>
+  </si>
+  <si>
+    <t>دل که سفره نیست که پیش همه پهنش کنی.</t>
+  </si>
+  <si>
+    <t>خرسو به آهنگری بسَّن.</t>
+  </si>
+  <si>
+    <t>ای آبُ تو هوَنگ کنه که بوکوبی، نَمی‌ذاره بیکار باشی.</t>
+  </si>
+  <si>
+    <t>کور اَی بازار نره بازار می‌گنده.</t>
+  </si>
+  <si>
+    <t>آیت کارت آخره.</t>
+  </si>
+  <si>
+    <t>چاکَن همیشه تهِ چاهه.</t>
+  </si>
+  <si>
+    <t>قیمت غذا نسبت به حجم غذا خیلی خیلی گرون و غیرمنصفانه‌ن. ساندویچ هیولُی ژامبون در حد یِی بچه غولی هم نبود و اصلاً هم خوشمزه نبود اما ساندویچ چوریتسو عالی و بسیار بسیار خوشمزه بود.</t>
+  </si>
+  <si>
+    <t>لطف کنید از عکسوی اینترنتی استفاده نکنید و عکس خود محصولتونه بذارین. آخه ای کجو و او کجو. متأسفم.</t>
+  </si>
+  <si>
+    <t>حجم ساندویچش کلاً نصف شده!</t>
+  </si>
+  <si>
+    <t>فوق‌العاده بی‌نمک بود و بوی تند گوشت می‌داد.</t>
+  </si>
+  <si>
+    <t>اول ایکه بوی بدی دُشت دوم ایکه به همه چی می‌خورد به جز رست بیف جوری که منو یاد گوشت آبپز داخل آبگوشت انداخت خیلی خیس بود نون خشک و بدمزه‌ای دُشت لطفاً تناسب مایعاته رعایت کنین احتمالاً آخرین باره که از اینجو سفارش می‌دم.</t>
+  </si>
+  <si>
+    <t>خو پَ چرو نمیوی؟</t>
+  </si>
+  <si>
+    <t>چاقوی تیز برِی بره نر اومده.</t>
+  </si>
+  <si>
+    <t>برِی خودت بخور، برِی مردم بوپوش.</t>
+  </si>
+  <si>
+    <t>سفره بابوی شُمو سر کوچه‌ن.</t>
+  </si>
+  <si>
+    <t>خدا خره دید بهش شاخ نداد</t>
+  </si>
+  <si>
+    <t>طرف ماره کشته، بچِی ماره زنده گُذُشته.</t>
+  </si>
+  <si>
+    <t>گند بخوره به کارت.</t>
+  </si>
+  <si>
+    <t>چشم زمسّون کوره.</t>
+  </si>
+  <si>
+    <t>انگُ اوره خانُم زُیده ما رِ کنیز.</t>
+  </si>
+  <si>
+    <t>می‌خواما یخه‌مه پاره کنم</t>
+  </si>
+  <si>
+    <t>زودی باش / دس بجنبون</t>
   </si>
 </sst>
 </file>
@@ -1316,11 +1433,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2467,15 +2584,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="27.6" customHeight="1">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
     </row>
     <row r="2" spans="1:10" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -2532,10 +2649,6 @@
       <c r="H3" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="I3" s="1">
-        <f>COUNTBLANK(H3:H102)</f>
-        <v>42</v>
-      </c>
     </row>
     <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="6" t="s">
@@ -2663,8 +2776,8 @@
       <c r="G8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="12" t="s">
-        <v>282</v>
+      <c r="H8" s="11" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2872,7 +2985,7 @@
         <v>48</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -2924,7 +3037,7 @@
         <v>41</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -3002,7 +3115,7 @@
         <v>41</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -3028,7 +3141,7 @@
         <v>41</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -3131,6 +3244,9 @@
       <c r="G26" s="8" t="s">
         <v>74</v>
       </c>
+      <c r="H26" s="1" t="s">
+        <v>294</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="6" t="s">
@@ -3154,6 +3270,9 @@
       <c r="G27" s="8" t="s">
         <v>74</v>
       </c>
+      <c r="H27" s="1" t="s">
+        <v>295</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="6" t="s">
@@ -3178,7 +3297,7 @@
         <v>79</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -3229,6 +3348,9 @@
       <c r="G30" s="8" t="s">
         <v>66</v>
       </c>
+      <c r="H30" s="1" t="s">
+        <v>296</v>
+      </c>
     </row>
     <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="6" t="s">
@@ -3252,6 +3374,9 @@
       <c r="G31" s="8" t="s">
         <v>66</v>
       </c>
+      <c r="H31" s="1" t="s">
+        <v>297</v>
+      </c>
     </row>
     <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="6" t="s">
@@ -3275,8 +3400,11 @@
       <c r="G32" s="8" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H32" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="6" t="s">
         <v>89</v>
       </c>
@@ -3298,8 +3426,11 @@
       <c r="G33" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H33" s="1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="6" t="s">
         <v>89</v>
       </c>
@@ -3321,8 +3452,11 @@
       <c r="G34" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H34" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="6" t="s">
         <v>89</v>
       </c>
@@ -3344,8 +3478,11 @@
       <c r="G35" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H35" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="6" t="s">
         <v>89</v>
       </c>
@@ -3367,8 +3504,11 @@
       <c r="G36" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H36" s="1" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="6" t="s">
         <v>89</v>
       </c>
@@ -3390,8 +3530,11 @@
       <c r="G37" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H37" s="1" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="6" t="s">
         <v>89</v>
       </c>
@@ -3413,8 +3556,11 @@
       <c r="G38" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H38" s="1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="6" t="s">
         <v>89</v>
       </c>
@@ -3436,8 +3582,11 @@
       <c r="G39" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H39" s="1" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="6" t="s">
         <v>89</v>
       </c>
@@ -3459,8 +3608,11 @@
       <c r="G40" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H40" s="1" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="6" t="s">
         <v>89</v>
       </c>
@@ -3482,8 +3634,11 @@
       <c r="G41" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" ht="20.100000000000001" customHeight="1">
+      <c r="H41" s="1" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="6" t="s">
         <v>89</v>
       </c>
@@ -3505,8 +3660,11 @@
       <c r="G42" s="8" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" ht="35.549999999999997" customHeight="1">
+      <c r="H42" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A43" s="6" t="s">
         <v>113</v>
       </c>
@@ -3528,8 +3686,11 @@
       <c r="G43" s="8" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" ht="35.549999999999997" customHeight="1">
+      <c r="H43" s="1" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A44" s="6" t="s">
         <v>113</v>
       </c>
@@ -3551,8 +3712,11 @@
       <c r="G44" s="8" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" ht="35.549999999999997" customHeight="1">
+      <c r="H44" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A45" s="6" t="s">
         <v>113</v>
       </c>
@@ -3574,8 +3738,11 @@
       <c r="G45" s="8" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" ht="35.549999999999997" customHeight="1">
+      <c r="H45" s="1" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A46" s="6" t="s">
         <v>113</v>
       </c>
@@ -3597,8 +3764,11 @@
       <c r="G46" s="8" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" ht="35.549999999999997" customHeight="1">
+      <c r="H46" s="1" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A47" s="6" t="s">
         <v>113</v>
       </c>
@@ -3620,8 +3790,11 @@
       <c r="G47" s="8" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" ht="35.549999999999997" customHeight="1">
+      <c r="H47" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A48" s="6" t="s">
         <v>113</v>
       </c>
@@ -3642,6 +3815,9 @@
       </c>
       <c r="G48" s="8" t="s">
         <v>118</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="35.549999999999997" customHeight="1">
@@ -3666,6 +3842,9 @@
       <c r="G49" s="8" t="s">
         <v>118</v>
       </c>
+      <c r="H49" s="1" t="s">
+        <v>314</v>
+      </c>
     </row>
     <row r="50" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A50" s="6" t="s">
@@ -3689,6 +3868,9 @@
       <c r="G50" s="8" t="s">
         <v>118</v>
       </c>
+      <c r="H50" s="1" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="51" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A51" s="6" t="s">
@@ -3712,6 +3894,9 @@
       <c r="G51" s="8" t="s">
         <v>118</v>
       </c>
+      <c r="H51" s="1" t="s">
+        <v>316</v>
+      </c>
     </row>
     <row r="52" spans="1:8" ht="35.549999999999997" customHeight="1">
       <c r="A52" s="6" t="s">
@@ -3735,6 +3920,9 @@
       <c r="G52" s="8" t="s">
         <v>118</v>
       </c>
+      <c r="H52" s="1" t="s">
+        <v>317</v>
+      </c>
     </row>
     <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A53" s="6" t="s">
@@ -3758,6 +3946,9 @@
       <c r="G53" s="8" t="s">
         <v>139</v>
       </c>
+      <c r="H53" s="1" t="s">
+        <v>318</v>
+      </c>
     </row>
     <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A54" s="6" t="s">
@@ -3781,6 +3972,9 @@
       <c r="G54" s="8" t="s">
         <v>139</v>
       </c>
+      <c r="H54" s="1" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="6" t="s">
@@ -3908,6 +4102,9 @@
       <c r="G59" s="8" t="s">
         <v>139</v>
       </c>
+      <c r="H59" s="1" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="60" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A60" s="6" t="s">
@@ -3957,6 +4154,9 @@
       <c r="G61" s="8" t="s">
         <v>139</v>
       </c>
+      <c r="H61" s="1" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="62" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A62" s="6" t="s">
@@ -3980,6 +4180,9 @@
       <c r="G62" s="8" t="s">
         <v>139</v>
       </c>
+      <c r="H62" s="1" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="63" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A63" s="6" t="s">
@@ -4033,7 +4236,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="65" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A65" s="6" t="s">
         <v>113</v>
       </c>
@@ -4055,11 +4258,11 @@
       <c r="G65" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="I65" s="1" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="H65" s="1" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A66" s="6" t="s">
         <v>113</v>
       </c>
@@ -4082,10 +4285,10 @@
         <v>159</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="20.100000000000001" customHeight="1">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A67" s="6" t="s">
         <v>113</v>
       </c>
@@ -4108,10 +4311,10 @@
         <v>159</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="20.100000000000001" customHeight="1">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A68" s="6" t="s">
         <v>113</v>
       </c>
@@ -4137,7 +4340,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="69" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A69" s="6" t="s">
         <v>113</v>
       </c>
@@ -4163,7 +4366,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="70" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A70" s="6" t="s">
         <v>113</v>
       </c>
@@ -4186,10 +4389,10 @@
         <v>152</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" ht="20.100000000000001" customHeight="1">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A71" s="6" t="s">
         <v>113</v>
       </c>
@@ -4211,8 +4414,11 @@
       <c r="G71" s="8" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" ht="20.100000000000001" customHeight="1">
+      <c r="H71" s="1" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A72" s="6" t="s">
         <v>113</v>
       </c>
@@ -4235,10 +4441,10 @@
         <v>159</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" ht="20.100000000000001" customHeight="1">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A73" s="6" t="s">
         <v>113</v>
       </c>
@@ -4260,11 +4466,11 @@
       <c r="G73" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H73" s="8" t="s">
+      <c r="H73" s="1" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="74" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A74" s="6" t="s">
         <v>113</v>
       </c>
@@ -4286,11 +4492,11 @@
       <c r="G74" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H74" s="8" t="s">
+      <c r="H74" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="75" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A75" s="6" t="s">
         <v>113</v>
       </c>
@@ -4312,11 +4518,11 @@
       <c r="G75" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H75" s="8" t="s">
+      <c r="H75" s="1" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="76" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A76" s="6" t="s">
         <v>113</v>
       </c>
@@ -4338,11 +4544,11 @@
       <c r="G76" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="H76" s="8" t="s">
+      <c r="H76" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="77" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A77" s="6" t="s">
         <v>113</v>
       </c>
@@ -4364,11 +4570,11 @@
       <c r="G77" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="H77" s="8" t="s">
+      <c r="H77" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="78" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A78" s="6" t="s">
         <v>113</v>
       </c>
@@ -4390,11 +4596,11 @@
       <c r="G78" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="H78" s="8" t="s">
+      <c r="H78" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="79" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A79" s="6" t="s">
         <v>113</v>
       </c>
@@ -4416,11 +4622,11 @@
       <c r="G79" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H79" s="8" t="s">
+      <c r="H79" s="1" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="20.100000000000001" customHeight="1">
+    <row r="80" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A80" s="6" t="s">
         <v>113</v>
       </c>
@@ -4442,7 +4648,7 @@
       <c r="G80" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H80" s="8" t="s">
+      <c r="H80" s="1" t="s">
         <v>190</v>
       </c>
     </row>
@@ -4468,7 +4674,7 @@
       <c r="G81" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H81" s="8" t="s">
+      <c r="H81" s="1" t="s">
         <v>192</v>
       </c>
     </row>
@@ -4494,7 +4700,7 @@
       <c r="G82" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H82" s="8" t="s">
+      <c r="H82" s="1" t="s">
         <v>194</v>
       </c>
     </row>
@@ -4520,6 +4726,9 @@
       <c r="G83" s="8" t="s">
         <v>199</v>
       </c>
+      <c r="H83" s="1" t="s">
+        <v>324</v>
+      </c>
     </row>
     <row r="84" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A84" s="6" t="s">
@@ -4543,6 +4752,9 @@
       <c r="G84" s="8" t="s">
         <v>199</v>
       </c>
+      <c r="H84" s="1" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="85" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A85" s="6" t="s">
@@ -4566,6 +4778,9 @@
       <c r="G85" s="8" t="s">
         <v>204</v>
       </c>
+      <c r="H85" s="1" t="s">
+        <v>326</v>
+      </c>
     </row>
     <row r="86" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A86" s="6" t="s">
@@ -4590,7 +4805,7 @@
         <v>207</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4616,7 +4831,7 @@
         <v>207</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4641,6 +4856,9 @@
       <c r="G88" s="8" t="s">
         <v>212</v>
       </c>
+      <c r="H88" s="1" t="s">
+        <v>327</v>
+      </c>
     </row>
     <row r="89" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A89" s="6" t="s">
@@ -4664,6 +4882,9 @@
       <c r="G89" s="8" t="s">
         <v>204</v>
       </c>
+      <c r="H89" s="1" t="s">
+        <v>328</v>
+      </c>
     </row>
     <row r="90" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A90" s="6" t="s">
@@ -4687,6 +4908,9 @@
       <c r="G90" s="8" t="s">
         <v>199</v>
       </c>
+      <c r="H90" s="1" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="91" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A91" s="6" t="s">
@@ -4710,6 +4934,9 @@
       <c r="G91" s="8" t="s">
         <v>199</v>
       </c>
+      <c r="H91" s="1" t="s">
+        <v>330</v>
+      </c>
     </row>
     <row r="92" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A92" s="6" t="s">
@@ -4734,7 +4961,7 @@
         <v>199</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4760,7 +4987,7 @@
         <v>41</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4786,7 +5013,7 @@
         <v>41</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4811,6 +5038,9 @@
       <c r="G95" s="8" t="s">
         <v>41</v>
       </c>
+      <c r="H95" s="11" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="96" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A96" s="6" t="s">
@@ -4835,7 +5065,7 @@
         <v>41</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4861,7 +5091,7 @@
         <v>233</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4887,7 +5117,7 @@
         <v>236</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4913,7 +5143,7 @@
         <v>239</v>
       </c>
       <c r="H99" s="1" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4938,6 +5168,9 @@
       <c r="G100" s="8" t="s">
         <v>242</v>
       </c>
+      <c r="H100" s="1" t="s">
+        <v>332</v>
+      </c>
     </row>
     <row r="101" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A101" s="6" t="s">
@@ -4961,6 +5194,9 @@
       <c r="G101" s="8" t="s">
         <v>41</v>
       </c>
+      <c r="H101" s="1" t="s">
+        <v>329</v>
+      </c>
     </row>
     <row r="102" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A102" s="6" t="s">
@@ -4985,7 +5221,7 @@
         <v>41</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Shirazi transliterations and update some Shirazi translations
The rows containing star (*) has "eh" in some words meaning "ast" or "raa".
</commit_message>
<xml_diff>
--- a/datasets/100_samples_shirazi.xlsx
+++ b/datasets/100_samples_shirazi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Personal Projects\SilkRoadNLP\Repositories\General\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA537B3C-BD87-4126-A5F3-0A8D5D9C0D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADD8B71-80E9-483E-BACC-E5F73E4ACA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="334">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="435">
   <si>
     <t>100_samples</t>
   </si>
@@ -978,9 +978,6 @@
     <t>خرس بخورتش می‌پوکه.</t>
   </si>
   <si>
-    <t>من چوی نَمی‌خورم</t>
-  </si>
-  <si>
     <t>عالی بود؛ بوس به جونت، قربونت برم</t>
   </si>
   <si>
@@ -1005,9 +1002,6 @@
     <t>تو کل عمرُم همچی غذاهوی نخوردم</t>
   </si>
   <si>
-    <t>دسِّتون درد نکنه بری پخش ای کلیپ درباره گیوه هرسینی</t>
-  </si>
-  <si>
     <t>بیشترشونو اولین باره می‌بینم</t>
   </si>
   <si>
@@ -1032,54 +1026,27 @@
     <t>جوی کیک وانیلی کاکائویی، کیک کاکايویی ساده ارسال شده بود.</t>
   </si>
   <si>
-    <t>خورشش مزِی آب می‌داد و ۹۵ درصد حجم قیمه‌ش لپه بود. اصلا پیشنهاد نَمی‌کنم.</t>
-  </si>
-  <si>
     <t>خیلی عالی و به‌موقع. ممنون از شُمو.</t>
   </si>
   <si>
-    <t>عالی. فقط جوی یِی چنگالی خالی بود</t>
-  </si>
-  <si>
     <t>پس چرو نَمیوی؟</t>
   </si>
   <si>
     <t>ما عَم میویم.</t>
   </si>
   <si>
-    <t>پس کجویی عزیزُم؟</t>
-  </si>
-  <si>
-    <t>بیو بریم ناهار بخوریم. وُی نه، یِی چی آشغالی خوردم، دلُم ریخته به هم.</t>
-  </si>
-  <si>
     <t>پنج و چار و سه</t>
   </si>
   <si>
     <t>کَمَرُم پُکید.</t>
   </si>
   <si>
-    <t>ای شکوفه‌ها چه قشنگن.</t>
-  </si>
-  <si>
     <t>خونِی شومو.</t>
   </si>
   <si>
-    <t>قدوی سرت. عیبی نداره.</t>
-  </si>
-  <si>
-    <t>خانوم بچه‌ها چیطورن؟</t>
-  </si>
-  <si>
-    <t>ای داد و بیداد برای میراث پدرامون که بی پشت و پنا موندن</t>
-  </si>
-  <si>
     <t>درود فراوون به زنوی کورد سر تا سر دنیا از کرمونشا گرفته تا کردستان</t>
   </si>
   <si>
-    <t>هر وقت نون درست می‌کِرد صدامون می‌زد. ما بچّا هم همگی به‌صف کنارش می‌شنسّیم و چشم به را می‌موندیم تا نون روی تووه برشته می‌شد و می‌داد دسّمون.</t>
-  </si>
-  <si>
     <t>او چیچیه که تا دس تو چیشش نکنی، چیلشه باز نَمی‌کنه؟</t>
   </si>
   <si>
@@ -1095,12 +1062,6 @@
     <t>عبده ای کی بود؟</t>
   </si>
   <si>
-    <t>تور خدا بفرمو داخل خونه.</t>
-  </si>
-  <si>
-    <t>دماغش چقد پهنه. لباش شبیه پشت میمونه.</t>
-  </si>
-  <si>
     <t>گربُو ره بُراق کِرده.</t>
   </si>
   <si>
@@ -1119,9 +1080,6 @@
     <t>خسّه</t>
   </si>
   <si>
-    <t>بوگو چقدر حال می‌ده</t>
-  </si>
-  <si>
     <t>لعنت به پدرت</t>
   </si>
   <si>
@@ -1137,18 +1095,9 @@
     <t>ما برِی تازه‌ترین آتیش منتظر می‌مونیم</t>
   </si>
   <si>
-    <t>یعنی ساخته نمی‌شه</t>
-  </si>
-  <si>
-    <t>با ایکه ده تو کارگر داره،‌ پونزده سال طول می‌کشه</t>
-  </si>
-  <si>
     <t>مِثکه کسوی دیگه‌ای هم با هواپیما به لوگر می‌رن</t>
   </si>
   <si>
-    <t>ساختن ای فرودگاهو هم عین رفتن به ماعه</t>
-  </si>
-  <si>
     <t>درخت میوه کرم از خودشه</t>
   </si>
   <si>
@@ -1161,9 +1110,6 @@
     <t>حرف تا وقتی تو دلته اختیارش دسِّته.</t>
   </si>
   <si>
-    <t>دل که سفره نیست که پیش همه پهنش کنی.</t>
-  </si>
-  <si>
     <t>خرسو به آهنگری بسَّن.</t>
   </si>
   <si>
@@ -1176,9 +1122,6 @@
     <t>آیت کارت آخره.</t>
   </si>
   <si>
-    <t>چاکَن همیشه تهِ چاهه.</t>
-  </si>
-  <si>
     <t>قیمت غذا نسبت به حجم غذا خیلی خیلی گرون و غیرمنصفانه‌ن. ساندویچ هیولُی ژامبون در حد یِی بچه غولی هم نبود و اصلاً هم خوشمزه نبود اما ساندویچ چوریتسو عالی و بسیار بسیار خوشمزه بود.</t>
   </si>
   <si>
@@ -1197,15 +1140,9 @@
     <t>خو پَ چرو نمیوی؟</t>
   </si>
   <si>
-    <t>چاقوی تیز برِی بره نر اومده.</t>
-  </si>
-  <si>
     <t>برِی خودت بخور، برِی مردم بوپوش.</t>
   </si>
   <si>
-    <t>سفره بابوی شُمو سر کوچه‌ن.</t>
-  </si>
-  <si>
     <t>خدا خره دید بهش شاخ نداد</t>
   </si>
   <si>
@@ -1224,14 +1161,390 @@
     <t>می‌خواما یخه‌مه پاره کنم</t>
   </si>
   <si>
-    <t>زودی باش / دس بجنبون</t>
+    <t>Dāram miram</t>
+  </si>
+  <si>
+    <t>Man choy namkhoram</t>
+  </si>
+  <si>
+    <t>من چوی نَمخورم</t>
+  </si>
+  <si>
+    <t>Āli bud; bus be junet, qorbunet beram</t>
+  </si>
+  <si>
+    <t>Emruz kojo daso rume shosse budam?</t>
+  </si>
+  <si>
+    <t>Ire khodā zadeh</t>
+  </si>
+  <si>
+    <t>Chi doros kerdi?</t>
+  </si>
+  <si>
+    <t>Dokhtarā dāran miran</t>
+  </si>
+  <si>
+    <t>Dokhtarā doshtan miraftan</t>
+  </si>
+  <si>
+    <t>Ravānshenāsā khavāse ziādi barey gerye kerdan dar ovordan va gerye kerdane barey rahā shodan az feshāre esteres va tahammole dardo ghamo ghose midunan.</t>
+  </si>
+  <si>
+    <t>U morabow khordan dāreh</t>
+  </si>
+  <si>
+    <t>خانوم بچّا چیطورن؟</t>
+  </si>
+  <si>
+    <t>Khanum bachchā chitoran?</t>
+  </si>
+  <si>
+    <t>دسِّتون درد نکنه بری پخش ای کیلیپ دربارِی گیوِی هرسینی</t>
+  </si>
+  <si>
+    <t>Dassetun dard nakoneh barey pakhshe i kilip darbārey givey harsini</t>
+  </si>
+  <si>
+    <t>Ey dādo bidād barey mirāse pedarāmun ke bi poshto pana mondan</t>
+  </si>
+  <si>
+    <t>ای داد و بیداد بری میراث پدرامون که بی پشت و پنا مُندن</t>
+  </si>
+  <si>
+    <t>Bishtareshuno avalin bāre mibinam</t>
+  </si>
+  <si>
+    <t>Ey junom barey shahremun</t>
+  </si>
+  <si>
+    <t>Dorude farāvun be zanoy korde sar tā sare donyā az kermunshā gerefte ta kordestān</t>
+  </si>
+  <si>
+    <t>Har vaght nun doros mikerd sedāmun mizad. Mā bachchā ham hamegi be saf kenāresh mishnessimo cheshm be rā mimondim tā nun ruye towe bereshte mishodo midād dassemun.</t>
+  </si>
+  <si>
+    <t>هر وقت نون دُرُس می‌کِرد صدامون می‌زد. ما بچّا هم همگی به‌صف کنارش می‌شنسّیم و چشم به را می‌مُندیم تا نون روی توه برشته می‌شد و می‌داد دسّمون.</t>
+  </si>
+  <si>
+    <t>Bordano ovordan</t>
+  </si>
+  <si>
+    <t>Dādo bidād</t>
+  </si>
+  <si>
+    <t>Khodā negadār</t>
+  </si>
+  <si>
+    <t>Ay amre hazrate haq nabāshe, barg az derakht namiofteh.</t>
+  </si>
+  <si>
+    <t>Ay nakhordim nune gandom, vali didim dasse mardom.</t>
+  </si>
+  <si>
+    <t>U chichieh keh tā das to chishesh nakoni, chileshe bāz namikoneh?</t>
+  </si>
+  <si>
+    <t>Mey behet zang nazadan?</t>
+  </si>
+  <si>
+    <t>Jār</t>
+  </si>
+  <si>
+    <t>Khasse</t>
+  </si>
+  <si>
+    <t>Farār</t>
+  </si>
+  <si>
+    <t>Tu kolle omrom hamchi ghazāhoy nakhordam</t>
+  </si>
+  <si>
+    <t>Bugu cheqad hāl mideh</t>
+  </si>
+  <si>
+    <t>بوگو چقد حال می‌ده</t>
+  </si>
+  <si>
+    <t>La‘nat be pedaret</t>
+  </si>
+  <si>
+    <t>Hakeroy mā az hakeroy digeh chizi kam nadāran</t>
+  </si>
+  <si>
+    <t>Kheili jāleb misheh</t>
+  </si>
+  <si>
+    <t>Faghat voyso barey yeki az bāzioy bāhālet</t>
+  </si>
+  <si>
+    <t>Ma barey tāzetarin ātish montazer mimunim</t>
+  </si>
+  <si>
+    <t>یَنی ساخته نمی‌شه</t>
+  </si>
+  <si>
+    <t>Yani sakhteh namisheh</t>
+  </si>
+  <si>
+    <t>با ایکه دَ تو کارگر داره،‌ پونزَ سال طول می‌کشه</t>
+  </si>
+  <si>
+    <t>Bā ike da to kārgar dāreh, punza sāl tul mikeshe</t>
+  </si>
+  <si>
+    <t>Meske kasoy degei ham bā hāvāpeyma be logar miran</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Derakhte mive kerm az khodeshe</t>
+  </si>
+  <si>
+    <t>Birune bāgho ke didim, engo tā tahe bāgho didim.</t>
+  </si>
+  <si>
+    <t>Hareh ay dākhele shisheh koni beh birun darz mikoneh.</t>
+  </si>
+  <si>
+    <t>دل که سفره نیس که پیش همه پهنش کنی.</t>
+  </si>
+  <si>
+    <t>Del ke sofre nis ke pishe hame pahnesh koni.</t>
+  </si>
+  <si>
+    <t>Kherso be āhangari bassan.</t>
+  </si>
+  <si>
+    <t>Ay ābo tu howang koneh ke bukubi, namizāreh bikār bāshi.</t>
+  </si>
+  <si>
+    <t>Kur ay bāzār nareh bāzār migandeh.</t>
+  </si>
+  <si>
+    <t>Āyat kāret akhere.</t>
+  </si>
+  <si>
+    <t>Chākan hamisheh ta chāheh.</t>
+  </si>
+  <si>
+    <t>چاکَن همیشه تَ چاهه.</t>
+  </si>
+  <si>
+    <t>Qeymate ghazā nesbat beh hajme ghazā kheili geruno gheyremonsefānan. Sāndeviche hayuloy zhāmbon dar hadde yey bachche ghuli ham nabud va aslan ham khoshmazeh nabud ammā sandeviche choritso ālio besyār besyār khoshmazeh bud.</t>
+  </si>
+  <si>
+    <t>Lotf konid az aksoy interneti estefādeh nakonid va akse khode mahsuletuneh bezārin. Ākhe i kojo o u kojo. Mote’asefam.</t>
+  </si>
+  <si>
+    <t>Badjur āsib dideh bud (tebqe akse āplowdshodeh)</t>
+  </si>
+  <si>
+    <t>Joy keyke vanili kākā’ui, keyke kākā’uie sādeh ersal shodeh bud.</t>
+  </si>
+  <si>
+    <t>Khoreshesh mazzey āb midād va navado panj darsade hajme qeymash lappe bud. Aslan pishnāhād namikonam.</t>
+  </si>
+  <si>
+    <t>خورشش مزِّی آب می‌داد و نود و پنج درصد حجم قیمه‌ش لپّه بود. اصلا پیشناهاد نَمی‌کنم.</t>
+  </si>
+  <si>
+    <t>Kheili ālio bemoqeh. Mamnun az shomo.</t>
+  </si>
+  <si>
+    <t>Hajme sāndevichesh kollan nesf shode!</t>
+  </si>
+  <si>
+    <t>Āli. Faghat joy yey changāli khāali bud.</t>
+  </si>
+  <si>
+    <t>عالی. فقط جوی یِی چنگالی خالی بود.</t>
+  </si>
+  <si>
+    <t>Fogholādeh binamak bud va buye tonde gusht midād.</t>
+  </si>
+  <si>
+    <t>Aval ikeh buye bady dosht dovom ikeh beh hame chi mikhord beh joz rost bif juri keh mano yāde gushte ābpaz dākhele ābgusht endākht kheili khis bud nune khoshko badmazei dosht lotfan tanāsobe māye‘āte ra‘āyat konin ehtemālan ākherin bāre ke az injo sefāresh midam.</t>
+  </si>
+  <si>
+    <t>Pas chero namioy?</t>
+  </si>
+  <si>
+    <t>Ma am mioym.</t>
+  </si>
+  <si>
+    <t>Zudi bāsh / Das bojombun</t>
+  </si>
+  <si>
+    <t>زودی باش / دس بجمبون</t>
+  </si>
+  <si>
+    <t>Pas kojoi azizom</t>
+  </si>
+  <si>
+    <t>پس کُجُی عزیزُم؟</t>
+  </si>
+  <si>
+    <t>بیو بیریم ناهار بخوریم. وُی نه، یِی چی آشغالی خوردم، دلُم ریخته به هم.</t>
+  </si>
+  <si>
+    <t>Bio birim nāhār bokhorim. Voy na, yey chi āshghali khordam, delom rikhteh be ham.</t>
+  </si>
+  <si>
+    <t>Mano towo hasan</t>
+  </si>
+  <si>
+    <t>Golo bolbolo sonbol</t>
+  </si>
+  <si>
+    <t>Panjo chāro she</t>
+  </si>
+  <si>
+    <t>Kho pa chro namioy?</t>
+  </si>
+  <si>
+    <t>Kamarom pokid.</t>
+  </si>
+  <si>
+    <t>I kāru ke eqad osom osom kerdan nadāreh keh</t>
+  </si>
+  <si>
+    <t>Ye bār digeh ijuri besheh mikhābam tu kheresh</t>
+  </si>
+  <si>
+    <t>Az beh khub bud kompich gereftam</t>
+  </si>
+  <si>
+    <t>Vasey chi?</t>
+  </si>
+  <si>
+    <t>I khodesho bā shākhe gāv darendākhteh.</t>
+  </si>
+  <si>
+    <t>Khodā dune khadijeh</t>
+  </si>
+  <si>
+    <t>Hālo eqadam beshkano bālo bendāz khub ni</t>
+  </si>
+  <si>
+    <t>Mey dombālet gozoshtan?</t>
+  </si>
+  <si>
+    <r>
+      <t>Nune gandom, kome fulādi mikhā</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>d.</t>
+    </r>
+  </si>
+  <si>
+    <t>Ia nam tok pas namideh</t>
+  </si>
+  <si>
+    <t>چاقوی تیز برِی برِیِ نر اومده.</t>
+  </si>
+  <si>
+    <t>Chāquye tiz barey baareye nar umadeh.</t>
+  </si>
+  <si>
+    <t>Barey khodet bokhor, barey mardom bupush.</t>
+  </si>
+  <si>
+    <t>سُفرِی بابوی شُمو سر کوچه‌ن.</t>
+  </si>
+  <si>
+    <t>Sofrey bāboy shomo sar kuchan.</t>
+  </si>
+  <si>
+    <t>ای شوکوفه‌ها چه قشنگن.</t>
+  </si>
+  <si>
+    <t>I shukufeha che qashangan.</t>
+  </si>
+  <si>
+    <t>Khuney shomo.</t>
+  </si>
+  <si>
+    <t>Khodā khare did behesh shākh nadād</t>
+  </si>
+  <si>
+    <t>Taraf māreh koshteh, bachey māreh zendeh gozoshteh.</t>
+  </si>
+  <si>
+    <t>Jangali shotor dideh.</t>
+  </si>
+  <si>
+    <t>Cheshme zemessun kureh.</t>
+  </si>
+  <si>
+    <t>Gorbow reh borāq kerdeh.</t>
+  </si>
+  <si>
+    <t>فدوی سرت. عیبی نداره.</t>
+  </si>
+  <si>
+    <t>Fadoy saret. Eibi nadāreh.</t>
+  </si>
+  <si>
+    <t>دماغش چقد پَنه. لباش شبی پشت میمونه.</t>
+  </si>
+  <si>
+    <t>Damāghesh cheqad paaneh. Labāsh shabi posthe meymuneh.</t>
+  </si>
+  <si>
+    <t>Engo ureh khānom zoydeh māa reh kaniz.</t>
+  </si>
+  <si>
+    <t>Abdeh i ki bud?</t>
+  </si>
+  <si>
+    <t>Gholām bā abre sia umado dokhtareh beh qasre shāhe pariun bord.</t>
+  </si>
+  <si>
+    <t>I viu cheqad qashangeh.</t>
+  </si>
+  <si>
+    <t>Mikhāma yakhame pāreh konam</t>
+  </si>
+  <si>
+    <t>Gand bokhoreh beh kāret.</t>
+  </si>
+  <si>
+    <t>Barakse mādaresh ke āqel bud khodesh engo diunan.</t>
+  </si>
+  <si>
+    <t>Goshnameh</t>
+  </si>
+  <si>
+    <t>Khers bokhoratesh mipokeh.</t>
+  </si>
+  <si>
+    <t>Harf tā vaqti tu deleteh ekhtiāresh dasseteh.</t>
+  </si>
+  <si>
+    <t>Tor khodā befarmo tu khuneh.</t>
+  </si>
+  <si>
+    <t>تور خدا بفرمو تو خونه.</t>
+  </si>
+  <si>
+    <t>Sākhtane i furudgowam eine raftan be māheh</t>
+  </si>
+  <si>
+    <t>ساختن ای فورودگوَم عین رفتن به ماهه</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -1258,6 +1571,12 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1399,7 +1718,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1438,6 +1757,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2579,7 +2901,7 @@
     <col min="6" max="6" width="84.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="102.33203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="30" style="1" customWidth="1"/>
+    <col min="9" max="9" width="71.33203125" style="1" customWidth="1"/>
     <col min="10" max="16384" width="8.33203125" style="1"/>
   </cols>
   <sheetData>
@@ -2649,6 +2971,9 @@
       <c r="H3" s="1" t="s">
         <v>249</v>
       </c>
+      <c r="I3" s="1" t="s">
+        <v>312</v>
+      </c>
     </row>
     <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="6" t="s">
@@ -2675,6 +3000,9 @@
       <c r="H4" s="1" t="s">
         <v>250</v>
       </c>
+      <c r="I4" s="1" t="s">
+        <v>429</v>
+      </c>
     </row>
     <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="6" t="s">
@@ -2701,6 +3029,12 @@
       <c r="H5" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="I5" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="6" t="s">
@@ -2725,7 +3059,10 @@
         <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>251</v>
+        <v>314</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2751,7 +3088,10 @@
         <v>25</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2777,7 +3117,10 @@
         <v>17</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>293</v>
+        <v>280</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2803,7 +3146,10 @@
         <v>17</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2829,7 +3175,10 @@
         <v>14</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2855,7 +3204,10 @@
         <v>34</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2881,7 +3233,10 @@
         <v>34</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>320</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2907,7 +3262,10 @@
         <v>41</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>257</v>
+        <v>256</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2933,7 +3291,10 @@
         <v>41</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2959,7 +3320,10 @@
         <v>41</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>259</v>
+        <v>258</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1">
@@ -2985,10 +3349,13 @@
         <v>48</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>323</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A17" s="6" t="s">
         <v>37</v>
       </c>
@@ -3011,10 +3378,13 @@
         <v>41</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>325</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="6" t="s">
         <v>37</v>
       </c>
@@ -3037,10 +3407,13 @@
         <v>41</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>328</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="6" t="s">
         <v>37</v>
       </c>
@@ -3063,10 +3436,13 @@
         <v>41</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>259</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="6" t="s">
         <v>37</v>
       </c>
@@ -3089,10 +3465,13 @@
         <v>41</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>260</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="6" t="s">
         <v>37</v>
       </c>
@@ -3115,10 +3494,13 @@
         <v>41</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>273</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="6" t="s">
         <v>37</v>
       </c>
@@ -3141,10 +3523,13 @@
         <v>41</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>333</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="6" t="s">
         <v>61</v>
       </c>
@@ -3167,10 +3552,13 @@
         <v>66</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>261</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A24" s="6" t="s">
         <v>61</v>
       </c>
@@ -3193,10 +3581,13 @@
         <v>66</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>262</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A25" s="6" t="s">
         <v>61</v>
       </c>
@@ -3219,10 +3610,13 @@
         <v>71</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>263</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A26" s="6" t="s">
         <v>61</v>
       </c>
@@ -3245,10 +3639,13 @@
         <v>74</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>281</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A27" s="6" t="s">
         <v>61</v>
       </c>
@@ -3271,10 +3668,13 @@
         <v>74</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>282</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A28" s="6" t="s">
         <v>61</v>
       </c>
@@ -3297,10 +3697,13 @@
         <v>79</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>274</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A29" s="6" t="s">
         <v>61</v>
       </c>
@@ -3323,10 +3726,13 @@
         <v>82</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>264</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A30" s="6" t="s">
         <v>61</v>
       </c>
@@ -3349,10 +3755,13 @@
         <v>66</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>283</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A31" s="6" t="s">
         <v>61</v>
       </c>
@@ -3375,10 +3784,13 @@
         <v>66</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>284</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A32" s="6" t="s">
         <v>61</v>
       </c>
@@ -3403,8 +3815,11 @@
       <c r="H32" s="1" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I32" s="1" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="6" t="s">
         <v>89</v>
       </c>
@@ -3427,10 +3842,13 @@
         <v>94</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>346</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="6" t="s">
         <v>89</v>
       </c>
@@ -3453,10 +3871,13 @@
         <v>94</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>285</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="6" t="s">
         <v>89</v>
       </c>
@@ -3479,10 +3900,13 @@
         <v>94</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>286</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="6" t="s">
         <v>89</v>
       </c>
@@ -3505,10 +3929,13 @@
         <v>94</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>287</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="6" t="s">
         <v>89</v>
       </c>
@@ -3531,10 +3958,13 @@
         <v>94</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>288</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="6" t="s">
         <v>89</v>
       </c>
@@ -3557,10 +3987,13 @@
         <v>94</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>289</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="6" t="s">
         <v>89</v>
       </c>
@@ -3583,10 +4016,13 @@
         <v>94</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>352</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="6" t="s">
         <v>89</v>
       </c>
@@ -3609,10 +4045,13 @@
         <v>94</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>354</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="6" t="s">
         <v>89</v>
       </c>
@@ -3635,10 +4074,13 @@
         <v>94</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>290</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="6" t="s">
         <v>89</v>
       </c>
@@ -3661,10 +4103,16 @@
         <v>94</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>434</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="J42" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A43" s="6" t="s">
         <v>113</v>
       </c>
@@ -3687,10 +4135,13 @@
         <v>118</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>291</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A44" s="6" t="s">
         <v>113</v>
       </c>
@@ -3713,10 +4164,13 @@
         <v>118</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>292</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A45" s="6" t="s">
         <v>113</v>
       </c>
@@ -3739,10 +4193,13 @@
         <v>118</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>293</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A46" s="6" t="s">
         <v>113</v>
       </c>
@@ -3765,10 +4222,16 @@
         <v>118</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>294</v>
+      </c>
+      <c r="I46" s="10" t="s">
+        <v>430</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A47" s="6" t="s">
         <v>113</v>
       </c>
@@ -3791,10 +4254,13 @@
         <v>118</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>361</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A48" s="6" t="s">
         <v>113</v>
       </c>
@@ -3817,10 +4283,13 @@
         <v>118</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>295</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A49" s="6" t="s">
         <v>113</v>
       </c>
@@ -3843,10 +4312,13 @@
         <v>118</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>296</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A50" s="6" t="s">
         <v>113</v>
       </c>
@@ -3869,10 +4341,13 @@
         <v>118</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>297</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A51" s="6" t="s">
         <v>113</v>
       </c>
@@ -3895,10 +4370,13 @@
         <v>118</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="35.549999999999997" customHeight="1">
+        <v>298</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="35.549999999999997" customHeight="1">
       <c r="A52" s="6" t="s">
         <v>113</v>
       </c>
@@ -3921,10 +4399,16 @@
         <v>118</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>368</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A53" s="6" t="s">
         <v>113</v>
       </c>
@@ -3947,10 +4431,13 @@
         <v>139</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>299</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A54" s="6" t="s">
         <v>113</v>
       </c>
@@ -3973,10 +4460,13 @@
         <v>139</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>300</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="6" t="s">
         <v>113</v>
       </c>
@@ -3999,10 +4489,13 @@
         <v>139</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>265</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="6" t="s">
         <v>113</v>
       </c>
@@ -4025,10 +4518,13 @@
         <v>139</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>266</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A57" s="6" t="s">
         <v>113</v>
       </c>
@@ -4051,10 +4547,13 @@
         <v>139</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>374</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A58" s="6" t="s">
         <v>113</v>
       </c>
@@ -4077,10 +4576,13 @@
         <v>139</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>267</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A59" s="6" t="s">
         <v>113</v>
       </c>
@@ -4103,10 +4605,13 @@
         <v>139</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>301</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A60" s="6" t="s">
         <v>113</v>
       </c>
@@ -4129,10 +4634,13 @@
         <v>139</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>378</v>
+      </c>
+      <c r="I60" s="13" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A61" s="6" t="s">
         <v>113</v>
       </c>
@@ -4155,10 +4663,13 @@
         <v>139</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>302</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A62" s="6" t="s">
         <v>113</v>
       </c>
@@ -4181,10 +4692,13 @@
         <v>139</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>303</v>
+      </c>
+      <c r="I62" s="10" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A63" s="6" t="s">
         <v>113</v>
       </c>
@@ -4207,10 +4721,13 @@
         <v>152</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>268</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A64" s="6" t="s">
         <v>113</v>
       </c>
@@ -4233,10 +4750,13 @@
         <v>152</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>269</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A65" s="6" t="s">
         <v>113</v>
       </c>
@@ -4259,10 +4779,13 @@
         <v>152</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>384</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A66" s="6" t="s">
         <v>113</v>
       </c>
@@ -4285,10 +4808,13 @@
         <v>159</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>386</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A67" s="6" t="s">
         <v>113</v>
       </c>
@@ -4311,10 +4837,13 @@
         <v>159</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>387</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A68" s="6" t="s">
         <v>113</v>
       </c>
@@ -4339,8 +4868,11 @@
       <c r="H68" s="1" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I68" s="1" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A69" s="6" t="s">
         <v>113</v>
       </c>
@@ -4365,8 +4897,11 @@
       <c r="H69" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I69" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A70" s="6" t="s">
         <v>113</v>
       </c>
@@ -4389,10 +4924,13 @@
         <v>152</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>270</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A71" s="6" t="s">
         <v>113</v>
       </c>
@@ -4415,10 +4953,13 @@
         <v>152</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>304</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A72" s="6" t="s">
         <v>113</v>
       </c>
@@ -4441,10 +4982,13 @@
         <v>159</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>271</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A73" s="6" t="s">
         <v>113</v>
       </c>
@@ -4469,8 +5013,11 @@
       <c r="H73" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I73" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A74" s="6" t="s">
         <v>113</v>
       </c>
@@ -4495,8 +5042,11 @@
       <c r="H74" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I74" s="1" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A75" s="6" t="s">
         <v>113</v>
       </c>
@@ -4521,8 +5071,11 @@
       <c r="H75" s="1" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I75" s="1" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A76" s="6" t="s">
         <v>113</v>
       </c>
@@ -4547,8 +5100,11 @@
       <c r="H76" s="1" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I76" s="1" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A77" s="6" t="s">
         <v>113</v>
       </c>
@@ -4573,8 +5129,11 @@
       <c r="H77" s="1" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I77" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A78" s="6" t="s">
         <v>113</v>
       </c>
@@ -4599,8 +5158,11 @@
       <c r="H78" s="1" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I78" s="1" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A79" s="6" t="s">
         <v>113</v>
       </c>
@@ -4625,8 +5187,11 @@
       <c r="H79" s="1" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I79" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A80" s="6" t="s">
         <v>113</v>
       </c>
@@ -4651,8 +5216,11 @@
       <c r="H80" s="1" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I80" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A81" s="6" t="s">
         <v>113</v>
       </c>
@@ -4677,8 +5245,11 @@
       <c r="H81" s="1" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I81" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A82" s="6" t="s">
         <v>113</v>
       </c>
@@ -4703,8 +5274,11 @@
       <c r="H82" s="1" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I82" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A83" s="6" t="s">
         <v>196</v>
       </c>
@@ -4727,10 +5301,13 @@
         <v>199</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>404</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A84" s="6" t="s">
         <v>196</v>
       </c>
@@ -4753,10 +5330,13 @@
         <v>199</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>305</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A85" s="6" t="s">
         <v>196</v>
       </c>
@@ -4779,10 +5359,13 @@
         <v>204</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>407</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A86" s="6" t="s">
         <v>196</v>
       </c>
@@ -4805,10 +5388,13 @@
         <v>207</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>409</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A87" s="6" t="s">
         <v>196</v>
       </c>
@@ -4831,10 +5417,13 @@
         <v>207</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>272</v>
+      </c>
+      <c r="I87" s="1" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A88" s="6" t="s">
         <v>196</v>
       </c>
@@ -4857,10 +5446,13 @@
         <v>212</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>306</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A89" s="6" t="s">
         <v>196</v>
       </c>
@@ -4883,10 +5475,16 @@
         <v>204</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="90" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>307</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="J89" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A90" s="6" t="s">
         <v>196</v>
       </c>
@@ -4911,8 +5509,11 @@
       <c r="H90" s="1" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" ht="20.100000000000001" customHeight="1">
+      <c r="I90" s="1" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A91" s="6" t="s">
         <v>196</v>
       </c>
@@ -4935,10 +5536,16 @@
         <v>199</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>309</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A92" s="6" t="s">
         <v>196</v>
       </c>
@@ -4961,10 +5568,16 @@
         <v>199</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>279</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A93" s="6" t="s">
         <v>221</v>
       </c>
@@ -4987,10 +5600,13 @@
         <v>41</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="94" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>417</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A94" s="6" t="s">
         <v>221</v>
       </c>
@@ -5013,10 +5629,16 @@
         <v>41</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>419</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="J94" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A95" s="6" t="s">
         <v>221</v>
       </c>
@@ -5039,10 +5661,13 @@
         <v>41</v>
       </c>
       <c r="H95" s="11" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="96" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>310</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A96" s="6" t="s">
         <v>221</v>
       </c>
@@ -5065,10 +5690,16 @@
         <v>41</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="97" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>432</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="J96" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A97" s="6" t="s">
         <v>221</v>
       </c>
@@ -5091,10 +5722,16 @@
         <v>233</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>278</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="J97" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A98" s="6" t="s">
         <v>221</v>
       </c>
@@ -5117,10 +5754,13 @@
         <v>236</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="99" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>277</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A99" s="6" t="s">
         <v>221</v>
       </c>
@@ -5143,10 +5783,13 @@
         <v>239</v>
       </c>
       <c r="H99" s="1" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="100" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>276</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A100" s="6" t="s">
         <v>221</v>
       </c>
@@ -5169,10 +5812,13 @@
         <v>242</v>
       </c>
       <c r="H100" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="101" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>311</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A101" s="6" t="s">
         <v>221</v>
       </c>
@@ -5195,10 +5841,13 @@
         <v>41</v>
       </c>
       <c r="H101" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="102" spans="1:8" ht="20.100000000000001" customHeight="1">
+        <v>308</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A102" s="6" t="s">
         <v>221</v>
       </c>
@@ -5221,7 +5870,10 @@
         <v>41</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>286</v>
+        <v>275</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>427</v>
       </c>
     </row>
   </sheetData>
@@ -5279,7 +5931,7 @@
     <hyperlink ref="G100" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
   </hyperlinks>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId49"/>
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>

</xml_diff>

<commit_message>
Fix some records in Shirazi and remove stars
Fix some translations and transliterations about "eh" + some minor changes. Remove stars from the last column.
</commit_message>
<xml_diff>
--- a/datasets/100_samples_shirazi.xlsx
+++ b/datasets/100_samples_shirazi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Personal Projects\SilkRoadNLP\Repositories\General\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADD8B71-80E9-483E-BACC-E5F73E4ACA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC55C64-C143-43D9-B2D8-0265DB653577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="920" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="436">
   <si>
     <t>100_samples</t>
   </si>
@@ -1095,9 +1095,6 @@
     <t>ما برِی تازه‌ترین آتیش منتظر می‌مونیم</t>
   </si>
   <si>
-    <t>مِثکه کسوی دیگه‌ای هم با هواپیما به لوگر می‌رن</t>
-  </si>
-  <si>
     <t>درخت میوه کرم از خودشه</t>
   </si>
   <si>
@@ -1188,9 +1185,6 @@
     <t>Dokhtarā doshtan miraftan</t>
   </si>
   <si>
-    <t>Ravānshenāsā khavāse ziādi barey gerye kerdan dar ovordan va gerye kerdane barey rahā shodan az feshāre esteres va tahammole dardo ghamo ghose midunan.</t>
-  </si>
-  <si>
     <t>U morabow khordan dāreh</t>
   </si>
   <si>
@@ -1218,9 +1212,6 @@
     <t>Ey junom barey shahremun</t>
   </si>
   <si>
-    <t>Dorude farāvun be zanoy korde sar tā sare donyā az kermunshā gerefte ta kordestān</t>
-  </si>
-  <si>
     <t>Har vaght nun doros mikerd sedāmun mizad. Mā bachchā ham hamegi be saf kenāresh mishnessimo cheshm be rā mimondim tā nun ruye towe bereshte mishodo midād dassemun.</t>
   </si>
   <si>
@@ -1284,36 +1275,21 @@
     <t>یَنی ساخته نمی‌شه</t>
   </si>
   <si>
-    <t>Yani sakhteh namisheh</t>
-  </si>
-  <si>
     <t>با ایکه دَ تو کارگر داره،‌ پونزَ سال طول می‌کشه</t>
   </si>
   <si>
     <t>Bā ike da to kārgar dāreh, punza sāl tul mikeshe</t>
   </si>
   <si>
-    <t>Meske kasoy degei ham bā hāvāpeyma be logar miran</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>Derakhte mive kerm az khodeshe</t>
   </si>
   <si>
     <t>Birune bāgho ke didim, engo tā tahe bāgho didim.</t>
   </si>
   <si>
-    <t>Hareh ay dākhele shisheh koni beh birun darz mikoneh.</t>
-  </si>
-  <si>
     <t>دل که سفره نیس که پیش همه پهنش کنی.</t>
   </si>
   <si>
-    <t>Del ke sofre nis ke pishe hame pahnesh koni.</t>
-  </si>
-  <si>
     <t>Kherso be āhangari bassan.</t>
   </si>
   <si>
@@ -1326,18 +1302,9 @@
     <t>Āyat kāret akhere.</t>
   </si>
   <si>
-    <t>Chākan hamisheh ta chāheh.</t>
-  </si>
-  <si>
     <t>چاکَن همیشه تَ چاهه.</t>
   </si>
   <si>
-    <t>Qeymate ghazā nesbat beh hajme ghazā kheili geruno gheyremonsefānan. Sāndeviche hayuloy zhāmbon dar hadde yey bachche ghuli ham nabud va aslan ham khoshmazeh nabud ammā sandeviche choritso ālio besyār besyār khoshmazeh bud.</t>
-  </si>
-  <si>
-    <t>Lotf konid az aksoy interneti estefādeh nakonid va akse khode mahsuletuneh bezārin. Ākhe i kojo o u kojo. Mote’asefam.</t>
-  </si>
-  <si>
     <t>Badjur āsib dideh bud (tebqe akse āplowdshodeh)</t>
   </si>
   <si>
@@ -1350,12 +1317,6 @@
     <t>خورشش مزِّی آب می‌داد و نود و پنج درصد حجم قیمه‌ش لپّه بود. اصلا پیشناهاد نَمی‌کنم.</t>
   </si>
   <si>
-    <t>Kheili ālio bemoqeh. Mamnun az shomo.</t>
-  </si>
-  <si>
-    <t>Hajme sāndevichesh kollan nesf shode!</t>
-  </si>
-  <si>
     <t>Āli. Faghat joy yey changāli khāali bud.</t>
   </si>
   <si>
@@ -1365,12 +1326,6 @@
     <t>Fogholādeh binamak bud va buye tonde gusht midād.</t>
   </si>
   <si>
-    <t>Aval ikeh buye bady dosht dovom ikeh beh hame chi mikhord beh joz rost bif juri keh mano yāde gushte ābpaz dākhele ābgusht endākht kheili khis bud nune khoshko badmazei dosht lotfan tanāsobe māye‘āte ra‘āyat konin ehtemālan ākherin bāre ke az injo sefāresh midam.</t>
-  </si>
-  <si>
-    <t>Pas chero namioy?</t>
-  </si>
-  <si>
     <t>Ma am mioym.</t>
   </si>
   <si>
@@ -1380,43 +1335,22 @@
     <t>زودی باش / دس بجمبون</t>
   </si>
   <si>
-    <t>Pas kojoi azizom</t>
-  </si>
-  <si>
     <t>پس کُجُی عزیزُم؟</t>
   </si>
   <si>
     <t>بیو بیریم ناهار بخوریم. وُی نه، یِی چی آشغالی خوردم، دلُم ریخته به هم.</t>
   </si>
   <si>
-    <t>Bio birim nāhār bokhorim. Voy na, yey chi āshghali khordam, delom rikhteh be ham.</t>
-  </si>
-  <si>
     <t>Mano towo hasan</t>
   </si>
   <si>
-    <t>Golo bolbolo sonbol</t>
-  </si>
-  <si>
-    <t>Panjo chāro she</t>
-  </si>
-  <si>
-    <t>Kho pa chro namioy?</t>
-  </si>
-  <si>
     <t>Kamarom pokid.</t>
   </si>
   <si>
     <t>I kāru ke eqad osom osom kerdan nadāreh keh</t>
   </si>
   <si>
-    <t>Ye bār digeh ijuri besheh mikhābam tu kheresh</t>
-  </si>
-  <si>
     <t>Az beh khub bud kompich gereftam</t>
-  </si>
-  <si>
-    <t>Vasey chi?</t>
   </si>
   <si>
     <t>I khodesho bā shākhe gāv darendākhteh.</t>
@@ -1444,9 +1378,6 @@
     </r>
   </si>
   <si>
-    <t>Ia nam tok pas namideh</t>
-  </si>
-  <si>
     <t>چاقوی تیز برِی برِیِ نر اومده.</t>
   </si>
   <si>
@@ -1474,70 +1405,142 @@
     <t>Khodā khare did behesh shākh nadād</t>
   </si>
   <si>
-    <t>Taraf māreh koshteh, bachey māreh zendeh gozoshteh.</t>
-  </si>
-  <si>
     <t>Jangali shotor dideh.</t>
   </si>
   <si>
-    <t>Cheshme zemessun kureh.</t>
-  </si>
-  <si>
-    <t>Gorbow reh borāq kerdeh.</t>
-  </si>
-  <si>
     <t>فدوی سرت. عیبی نداره.</t>
   </si>
   <si>
-    <t>Fadoy saret. Eibi nadāreh.</t>
-  </si>
-  <si>
     <t>دماغش چقد پَنه. لباش شبی پشت میمونه.</t>
   </si>
   <si>
-    <t>Damāghesh cheqad paaneh. Labāsh shabi posthe meymuneh.</t>
-  </si>
-  <si>
-    <t>Engo ureh khānom zoydeh māa reh kaniz.</t>
-  </si>
-  <si>
     <t>Abdeh i ki bud?</t>
   </si>
   <si>
-    <t>Gholām bā abre sia umado dokhtareh beh qasre shāhe pariun bord.</t>
-  </si>
-  <si>
-    <t>I viu cheqad qashangeh.</t>
-  </si>
-  <si>
-    <t>Mikhāma yakhame pāreh konam</t>
-  </si>
-  <si>
-    <t>Gand bokhoreh beh kāret.</t>
-  </si>
-  <si>
     <t>Barakse mādaresh ke āqel bud khodesh engo diunan.</t>
   </si>
   <si>
-    <t>Goshnameh</t>
-  </si>
-  <si>
     <t>Khers bokhoratesh mipokeh.</t>
   </si>
   <si>
-    <t>Harf tā vaqti tu deleteh ekhtiāresh dasseteh.</t>
-  </si>
-  <si>
     <t>Tor khodā befarmo tu khuneh.</t>
   </si>
   <si>
     <t>تور خدا بفرمو تو خونه.</t>
   </si>
   <si>
-    <t>Sākhtane i furudgowam eine raftan be māheh</t>
-  </si>
-  <si>
     <t>ساختن ای فورودگوَم عین رفتن به ماهه</t>
+  </si>
+  <si>
+    <t>Goshname</t>
+  </si>
+  <si>
+    <t>Ravānshenāsā khavāse ziādi barey geryeh kerdan dar ovordan va geryeh kerdane barey rahā shodan az feshāre esteres va tahammole dardo ghamo ghose midunan.</t>
+  </si>
+  <si>
+    <t>Dorude farāvun be zanoy korde sar tā sare donyā az kermunshā gerefteh ta kordestān</t>
+  </si>
+  <si>
+    <t>Yani sākhteh namisheh</t>
+  </si>
+  <si>
+    <t>مِثکه کسوی دیگِیِم با هواپیما به لوگر می‌رن</t>
+  </si>
+  <si>
+    <t>Meske kasoy degeiam bā hāvāpeyma be logar miran</t>
+  </si>
+  <si>
+    <t>Sākhtane i furudgowam eine raftan be māhe</t>
+  </si>
+  <si>
+    <t>Harfe ay dākhele shisheh koni be birun darz mikoneh.</t>
+  </si>
+  <si>
+    <t>Harf tā vaqti tu delete ekhtiāresh dassete.</t>
+  </si>
+  <si>
+    <t>Del ke sofreh nis ke pishe hameh pahnesh koni.</t>
+  </si>
+  <si>
+    <t>Chākan hamisheh ta chāhe.</t>
+  </si>
+  <si>
+    <t>Qeymate ghazā nesbat be hajme ghazā kheili geruno gheyremonsefānan. Sāndeviche hayuloy zhāmbon dar hadde yey bachcheh ghuli ham nabud va aslan ham khoshmazeh nabud ammā sandeviche choritso ālio besyār besyār khoshmazeh bud.</t>
+  </si>
+  <si>
+    <t>Lotf konid az aksoy interneti estefādeh nakonid va akse khode mahsuletune bezārin. Ākhe i kojo o u kojo. Mote’asefam.</t>
+  </si>
+  <si>
+    <t>Kheili ālio bemoqe‘. Mamnun az shomo.</t>
+  </si>
+  <si>
+    <t>Hajme sāndevichesh kollan nesf shodeh!</t>
+  </si>
+  <si>
+    <t>Aval ike buye badi dosht dovom ike be hame chi mikhord be joz rost bif juri ke mano yāde gushte ābpaz dākhele ābgusht endākht kheili khis bud nune khoshko badmazei dosht lotfan tanāsobe māye‘āte ra‘āyat konin ehtemālan ākherin bāre ke az injo sefāresh midam.</t>
+  </si>
+  <si>
+    <t>Pas chero namyoy?</t>
+  </si>
+  <si>
+    <t>Pas kojoy azizom</t>
+  </si>
+  <si>
+    <t>Bio birim nāhār bokhorim. Voy na, yey chi āshghāli khordam, delom rikhteh be ham.</t>
+  </si>
+  <si>
+    <t>گل و بلبل و سمبل</t>
+  </si>
+  <si>
+    <t>Golo bolbolo sombol</t>
+  </si>
+  <si>
+    <t>Panjo chāro seh</t>
+  </si>
+  <si>
+    <t>Kho pa chero namioy?</t>
+  </si>
+  <si>
+    <t>ای کارو که اقد اُسُم اُسُم کردن نداره که</t>
+  </si>
+  <si>
+    <t>Ye bār dige ijuri besheh mikhābam tu kheresh</t>
+  </si>
+  <si>
+    <t>Vāsey chi?</t>
+  </si>
+  <si>
+    <t>Iyā nam tok pas namideh</t>
+  </si>
+  <si>
+    <t>Taraf māre koshteh, bachey māre zendeh gozoshteh.</t>
+  </si>
+  <si>
+    <t>Cheshme zemessun kure.</t>
+  </si>
+  <si>
+    <t>Gorbow re borāq kerdeh.</t>
+  </si>
+  <si>
+    <t>Fadoy saret. Eybi nadāreh.</t>
+  </si>
+  <si>
+    <t>Damāghesh cheqad paane. Labāsh shabi poshte meymune.</t>
+  </si>
+  <si>
+    <t>Engo ure khānom zoydeh māa re kaniz.</t>
+  </si>
+  <si>
+    <t>Gholām bā abre siā umado dokhtare be qasre shāhe pariun bord.</t>
+  </si>
+  <si>
+    <t>I viu cheqad qashange.</t>
+  </si>
+  <si>
+    <t>Mikhāmā yakhame pāreh konam</t>
+  </si>
+  <si>
+    <t>Gand bokhoreh be kāret.</t>
   </si>
 </sst>
 </file>
@@ -1718,7 +1721,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1752,14 +1755,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2891,7 +2891,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J102"/>
+  <dimension ref="A1:I102"/>
   <sheetFormatPr defaultColWidth="8.33203125" defaultRowHeight="19.95" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1" customWidth="1"/>
@@ -2905,7 +2905,7 @@
     <col min="10" max="16384" width="8.33203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27.6" customHeight="1">
+    <row r="1" spans="1:9" ht="27.6" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -2916,7 +2916,7 @@
       <c r="F1" s="12"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="2" spans="1:10" ht="20.25" customHeight="1">
+    <row r="2" spans="1:9" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2944,9 +2944,8 @@
       <c r="I2" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="J2" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="20.25" customHeight="1">
+    </row>
+    <row r="3" spans="1:9" ht="20.25" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -2972,10 +2971,10 @@
         <v>249</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
@@ -3001,10 +3000,10 @@
         <v>250</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
@@ -3030,13 +3029,10 @@
         <v>19</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>428</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
@@ -3059,13 +3055,13 @@
         <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
@@ -3091,10 +3087,10 @@
         <v>251</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A8" s="6" t="s">
         <v>8</v>
       </c>
@@ -3116,14 +3112,14 @@
       <c r="G8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="1" t="s">
         <v>280</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A9" s="6" t="s">
         <v>8</v>
       </c>
@@ -3149,10 +3145,10 @@
         <v>252</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A10" s="6" t="s">
         <v>8</v>
       </c>
@@ -3178,10 +3174,10 @@
         <v>253</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
@@ -3207,10 +3203,10 @@
         <v>254</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A12" s="6" t="s">
         <v>8</v>
       </c>
@@ -3236,10 +3232,10 @@
         <v>255</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A13" s="6" t="s">
         <v>37</v>
       </c>
@@ -3265,10 +3261,10 @@
         <v>256</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A14" s="6" t="s">
         <v>37</v>
       </c>
@@ -3294,10 +3290,10 @@
         <v>257</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A15" s="6" t="s">
         <v>37</v>
       </c>
@@ -3323,10 +3319,10 @@
         <v>258</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A16" s="6" t="s">
         <v>37</v>
       </c>
@@ -3349,10 +3345,10 @@
         <v>48</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3378,10 +3374,10 @@
         <v>41</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3407,10 +3403,10 @@
         <v>41</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3439,7 +3435,7 @@
         <v>259</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3468,7 +3464,7 @@
         <v>260</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3497,7 +3493,7 @@
         <v>273</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>331</v>
+        <v>401</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3523,10 +3519,10 @@
         <v>41</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3555,7 +3551,7 @@
         <v>261</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3584,7 +3580,7 @@
         <v>262</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3613,7 +3609,7 @@
         <v>263</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3642,7 +3638,7 @@
         <v>281</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3671,7 +3667,7 @@
         <v>282</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3700,7 +3696,7 @@
         <v>274</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3729,7 +3725,7 @@
         <v>264</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3758,7 +3754,7 @@
         <v>283</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3787,7 +3783,7 @@
         <v>284</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -3816,10 +3812,10 @@
         <v>88</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A33" s="6" t="s">
         <v>89</v>
       </c>
@@ -3842,13 +3838,13 @@
         <v>94</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A34" s="6" t="s">
         <v>89</v>
       </c>
@@ -3874,10 +3870,10 @@
         <v>285</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A35" s="6" t="s">
         <v>89</v>
       </c>
@@ -3903,10 +3899,10 @@
         <v>286</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A36" s="6" t="s">
         <v>89</v>
       </c>
@@ -3932,10 +3928,10 @@
         <v>287</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A37" s="6" t="s">
         <v>89</v>
       </c>
@@ -3961,10 +3957,10 @@
         <v>288</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A38" s="6" t="s">
         <v>89</v>
       </c>
@@ -3990,10 +3986,10 @@
         <v>289</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A39" s="6" t="s">
         <v>89</v>
       </c>
@@ -4016,13 +4012,13 @@
         <v>94</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A40" s="6" t="s">
         <v>89</v>
       </c>
@@ -4045,13 +4041,13 @@
         <v>94</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A41" s="6" t="s">
         <v>89</v>
       </c>
@@ -4074,13 +4070,13 @@
         <v>94</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>290</v>
+        <v>403</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A42" s="6" t="s">
         <v>89</v>
       </c>
@@ -4103,16 +4099,13 @@
         <v>94</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>434</v>
+        <v>398</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="J42" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A43" s="6" t="s">
         <v>113</v>
       </c>
@@ -4135,13 +4128,13 @@
         <v>118</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A44" s="6" t="s">
         <v>113</v>
       </c>
@@ -4164,13 +4157,13 @@
         <v>118</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A45" s="6" t="s">
         <v>113</v>
       </c>
@@ -4193,13 +4186,13 @@
         <v>118</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A46" s="6" t="s">
         <v>113</v>
       </c>
@@ -4222,16 +4215,13 @@
         <v>118</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="J46" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A47" s="6" t="s">
         <v>113</v>
       </c>
@@ -4254,13 +4244,13 @@
         <v>118</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A48" s="6" t="s">
         <v>113</v>
       </c>
@@ -4283,13 +4273,13 @@
         <v>118</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A49" s="6" t="s">
         <v>113</v>
       </c>
@@ -4312,13 +4302,13 @@
         <v>118</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A50" s="6" t="s">
         <v>113</v>
       </c>
@@ -4341,13 +4331,13 @@
         <v>118</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A51" s="6" t="s">
         <v>113</v>
       </c>
@@ -4370,13 +4360,13 @@
         <v>118</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="35.549999999999997" customHeight="1">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="35.549999999999997" customHeight="1">
       <c r="A52" s="6" t="s">
         <v>113</v>
       </c>
@@ -4399,16 +4389,13 @@
         <v>118</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="J52" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A53" s="6" t="s">
         <v>113</v>
       </c>
@@ -4431,13 +4418,13 @@
         <v>139</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A54" s="6" t="s">
         <v>113</v>
       </c>
@@ -4460,13 +4447,13 @@
         <v>139</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A55" s="6" t="s">
         <v>113</v>
       </c>
@@ -4492,10 +4479,10 @@
         <v>265</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A56" s="6" t="s">
         <v>113</v>
       </c>
@@ -4521,10 +4508,10 @@
         <v>266</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A57" s="6" t="s">
         <v>113</v>
       </c>
@@ -4547,13 +4534,13 @@
         <v>139</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>374</v>
+        <v>363</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A58" s="6" t="s">
         <v>113</v>
       </c>
@@ -4579,10 +4566,10 @@
         <v>267</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A59" s="6" t="s">
         <v>113</v>
       </c>
@@ -4605,13 +4592,13 @@
         <v>139</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A60" s="6" t="s">
         <v>113</v>
       </c>
@@ -4634,13 +4621,13 @@
         <v>139</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>378</v>
-      </c>
-      <c r="I60" s="13" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>365</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A61" s="6" t="s">
         <v>113</v>
       </c>
@@ -4663,13 +4650,13 @@
         <v>139</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A62" s="6" t="s">
         <v>113</v>
       </c>
@@ -4692,13 +4679,13 @@
         <v>139</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A63" s="6" t="s">
         <v>113</v>
       </c>
@@ -4724,10 +4711,10 @@
         <v>268</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A64" s="6" t="s">
         <v>113</v>
       </c>
@@ -4753,7 +4740,7 @@
         <v>269</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>382</v>
+        <v>367</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4779,10 +4766,10 @@
         <v>152</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>384</v>
+        <v>369</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>383</v>
+        <v>368</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4808,10 +4795,10 @@
         <v>159</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>386</v>
+        <v>370</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>385</v>
+        <v>416</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4837,10 +4824,10 @@
         <v>159</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>387</v>
+        <v>371</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>388</v>
+        <v>417</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4869,7 +4856,7 @@
         <v>163</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>389</v>
+        <v>372</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4895,10 +4882,10 @@
         <v>152</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>165</v>
+        <v>418</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>390</v>
+        <v>419</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4927,7 +4914,7 @@
         <v>270</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>391</v>
+        <v>420</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4953,10 +4940,10 @@
         <v>152</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I71" s="1" t="s">
-        <v>392</v>
+        <v>421</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -4985,7 +4972,7 @@
         <v>271</v>
       </c>
       <c r="I72" s="1" t="s">
-        <v>393</v>
+        <v>373</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5011,10 +4998,10 @@
         <v>41</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>173</v>
+        <v>422</v>
       </c>
       <c r="I73" s="1" t="s">
-        <v>394</v>
+        <v>374</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5043,7 +5030,7 @@
         <v>175</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>395</v>
+        <v>423</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5072,7 +5059,7 @@
         <v>177</v>
       </c>
       <c r="I75" s="1" t="s">
-        <v>396</v>
+        <v>375</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5101,7 +5088,7 @@
         <v>179</v>
       </c>
       <c r="I76" s="1" t="s">
-        <v>397</v>
+        <v>424</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5130,7 +5117,7 @@
         <v>182</v>
       </c>
       <c r="I77" s="1" t="s">
-        <v>398</v>
+        <v>376</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5159,7 +5146,7 @@
         <v>185</v>
       </c>
       <c r="I78" s="1" t="s">
-        <v>399</v>
+        <v>377</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5188,7 +5175,7 @@
         <v>188</v>
       </c>
       <c r="I79" s="1" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="20.100000000000001" customHeight="1">
@@ -5217,10 +5204,10 @@
         <v>190</v>
       </c>
       <c r="I80" s="1" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A81" s="6" t="s">
         <v>113</v>
       </c>
@@ -5246,10 +5233,10 @@
         <v>192</v>
       </c>
       <c r="I81" s="1" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A82" s="6" t="s">
         <v>113</v>
       </c>
@@ -5275,10 +5262,10 @@
         <v>194</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A83" s="6" t="s">
         <v>196</v>
       </c>
@@ -5301,13 +5288,13 @@
         <v>199</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>404</v>
+        <v>381</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A84" s="6" t="s">
         <v>196</v>
       </c>
@@ -5330,13 +5317,13 @@
         <v>199</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A85" s="6" t="s">
         <v>196</v>
       </c>
@@ -5359,13 +5346,13 @@
         <v>204</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>407</v>
+        <v>384</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A86" s="6" t="s">
         <v>196</v>
       </c>
@@ -5388,13 +5375,13 @@
         <v>207</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>409</v>
+        <v>386</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A87" s="6" t="s">
         <v>196</v>
       </c>
@@ -5420,10 +5407,10 @@
         <v>272</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A88" s="6" t="s">
         <v>196</v>
       </c>
@@ -5446,13 +5433,13 @@
         <v>212</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A89" s="6" t="s">
         <v>196</v>
       </c>
@@ -5475,16 +5462,13 @@
         <v>204</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="J89" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A90" s="6" t="s">
         <v>196</v>
       </c>
@@ -5510,10 +5494,10 @@
         <v>216</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A91" s="6" t="s">
         <v>196</v>
       </c>
@@ -5536,16 +5520,13 @@
         <v>199</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="J91" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A92" s="6" t="s">
         <v>196</v>
       </c>
@@ -5571,13 +5552,10 @@
         <v>279</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="J92" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A93" s="6" t="s">
         <v>221</v>
       </c>
@@ -5600,13 +5578,13 @@
         <v>41</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>417</v>
+        <v>391</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A94" s="6" t="s">
         <v>221</v>
       </c>
@@ -5629,16 +5607,13 @@
         <v>41</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>419</v>
+        <v>392</v>
       </c>
       <c r="I94" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="J94" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A95" s="6" t="s">
         <v>221</v>
       </c>
@@ -5660,14 +5635,14 @@
       <c r="G95" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="H95" s="11" t="s">
-        <v>310</v>
+      <c r="H95" s="1" t="s">
+        <v>309</v>
       </c>
       <c r="I95" s="1" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A96" s="6" t="s">
         <v>221</v>
       </c>
@@ -5690,16 +5665,13 @@
         <v>41</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>432</v>
+        <v>397</v>
       </c>
       <c r="I96" s="1" t="s">
-        <v>431</v>
-      </c>
-      <c r="J96" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A97" s="6" t="s">
         <v>221</v>
       </c>
@@ -5725,13 +5697,10 @@
         <v>278</v>
       </c>
       <c r="I97" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="J97" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A98" s="6" t="s">
         <v>221</v>
       </c>
@@ -5757,10 +5726,10 @@
         <v>277</v>
       </c>
       <c r="I98" s="1" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A99" s="6" t="s">
         <v>221</v>
       </c>
@@ -5786,10 +5755,10 @@
         <v>276</v>
       </c>
       <c r="I99" s="1" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A100" s="6" t="s">
         <v>221</v>
       </c>
@@ -5812,13 +5781,13 @@
         <v>242</v>
       </c>
       <c r="H100" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I100" s="1" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A101" s="6" t="s">
         <v>221</v>
       </c>
@@ -5841,13 +5810,13 @@
         <v>41</v>
       </c>
       <c r="H101" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I101" s="1" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="102" spans="1:10" ht="20.100000000000001" customHeight="1">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A102" s="6" t="s">
         <v>221</v>
       </c>
@@ -5873,7 +5842,7 @@
         <v>275</v>
       </c>
       <c r="I102" s="1" t="s">
-        <v>427</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>